<commit_message>
unified the two models and used instantiate for precompiling the stan model
</commit_message>
<xml_diff>
--- a/inst/notebooks/makers_details.xlsx
+++ b/inst/notebooks/makers_details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24b25e554f22146a/Masters Class notes/AIMS Rwanda/Thesis Phase/Publication Phase/Refactoring MalReBay/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\SwissTPH-Ubuntu-24.04\home\golumo\GitRepos\MalReBay\inst\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{D403CC85-76BC-4478-A233-D1D2E70AF80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26417E7E-DC63-4EC6-BCA3-4C1AF67F6512}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A33DDC83-9ECF-47B4-A1E6-FF6326F77DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B200665-48F8-48D7-B17C-7D3B5710279D}"/>
+    <workbookView xWindow="0" yWindow="980" windowWidth="19380" windowHeight="9830" xr2:uid="{7B200665-48F8-48D7-B17C-7D3B5710279D}"/>
   </bookViews>
   <sheets>
     <sheet name="markers_info" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="45">
   <si>
     <t>marker_id</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>TRAP3</t>
+  </si>
+  <si>
+    <t>cpmp1</t>
   </si>
 </sst>
 </file>
@@ -539,15 +542,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43E4F913-EFD9-4818-926C-D0A818E637D6}">
-  <dimension ref="A1:D39"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.86328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -561,7 +564,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>313</v>
       </c>
@@ -575,7 +578,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>383</v>
       </c>
@@ -589,7 +592,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -603,7 +606,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -617,7 +620,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -631,7 +634,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -645,7 +648,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2490</v>
       </c>
@@ -659,7 +662,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -673,7 +676,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -687,7 +690,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -701,7 +704,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -715,7 +718,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -729,7 +732,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -743,7 +746,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -757,7 +760,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -771,7 +774,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -785,7 +788,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -799,7 +802,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -813,7 +816,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -827,7 +830,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -841,7 +844,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -855,7 +858,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -869,7 +872,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -883,7 +886,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -897,7 +900,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -911,7 +914,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -925,7 +928,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -939,7 +942,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -953,7 +956,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>31</v>
       </c>
@@ -967,7 +970,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -981,7 +984,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -995,7 +998,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -1009,7 +1012,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1023,7 +1026,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>36</v>
       </c>
@@ -1037,7 +1040,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -1051,7 +1054,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -1065,7 +1068,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1079,7 +1082,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -1090,6 +1093,20 @@
         <v>38</v>
       </c>
       <c r="D39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" t="s">
+        <v>38</v>
+      </c>
+      <c r="D40" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>